<commit_message>
Update flashcard content for clarity and accuracy
Corrected Spanish translations and multiple-choice options for flashcard 'm7_09' in `flashcards.ts`, and updated the corresponding Excel file `mazo_07_higiene.xlsx`.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: de849984-099f-49b2-9d46-edffa459c63e
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ae280521-5ef4-4db7-b5ec-ba3e05beb1f1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/efd0c2b9-faba-4dcd-a542-cac018800a89/de849984-099f-49b2-9d46-edffa459c63e/2zfo0Vc
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/client/src/data/raw/mazo_07_higiene.xlsx
+++ b/client/src/data/raw/mazo_07_higiene.xlsx
@@ -888,13 +888,13 @@
         <v>Voy a ayudarle a girarse.</v>
       </c>
       <c r="N9" t="str">
-        <v>Please hold the support rail.</v>
+        <v>Por favor, sujete el riel de soporte.</v>
       </c>
       <c r="O9" t="str">
-        <v>I am going to change the sheets.</v>
+        <v>Voy a ayudarle a levantarse.</v>
       </c>
       <c r="P9" t="str">
-        <v>I am going to help you turn.</v>
+        <v>Voy a ayudarle a girarse.</v>
       </c>
       <c r="Q9" t="str">
         <v>hygiene</v>

</xml_diff>